<commit_message>
Ordeno el proyecto y mejoro las visualizaciones
</commit_message>
<xml_diff>
--- a/Salidas/data_C_completa.xlsx
+++ b/Salidas/data_C_completa.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W100"/>
+  <dimension ref="A1:W99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="12" max="12" width="20.7109375" style="2" customWidth="1"/>
@@ -7160,21 +7160,21 @@
     </row>
     <row r="73">
       <c r="A73">
-        <v>17642208</v>
+        <v>24880822</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>GOMEZ</t>
+          <t>RAMIREZ</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SANDRA EDITH</t>
+          <t>MONICA ANDREA</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>De 45 a 65 años</t>
+          <t>De 35 a 44 años</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -7189,34 +7189,34 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Hepatitis virales</t>
+          <t>Banco de Sangre</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1b</t>
+          <t>Virus Hepatitis C, genotipo 1a</t>
         </is>
       </c>
       <c r="I73">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J73">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>2017-42</t>
+          <t>2018-45</t>
         </is>
       </c>
       <c r="L73" s="2">
-        <v>45406</v>
+        <v>43468</v>
       </c>
       <c r="M73" s="3">
-        <v>43027</v>
+        <v>43413</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>RIO GRANDE</t>
+          <t>USHUAIA</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -7246,17 +7246,17 @@
       </c>
       <c r="T73" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="U73" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SIN DATOS</t>
         </is>
       </c>
       <c r="V73" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="W73" t="inlineStr">
@@ -7267,26 +7267,26 @@
     </row>
     <row r="74">
       <c r="A74">
-        <v>24880822</v>
+        <v>18084570</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>RAMIREZ</t>
+          <t>PELAYES</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MONICA ANDREA</t>
+          <t>JOSE ALBERTO</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>De 35 a 44 años</t>
+          <t>De 45 a 65 años</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -7296,34 +7296,34 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Banco de Sangre</t>
+          <t>Hepatitis virales</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1a</t>
+          <t>Virus Hepatitis C, genotipo 1b</t>
         </is>
       </c>
       <c r="I74">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="J74">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>2018-45</t>
+          <t>2020-22</t>
         </is>
       </c>
       <c r="L74" s="2">
-        <v>43468</v>
+        <v>44178</v>
       </c>
       <c r="M74" s="3">
-        <v>43413</v>
+        <v>43980</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>USHUAIA</t>
+          <t>RIO GRANDE</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -7338,7 +7338,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -7348,17 +7348,17 @@
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="T74" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>SIN DATOS</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="V74" t="inlineStr">
@@ -7368,22 +7368,22 @@
       </c>
       <c r="W74" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75">
-        <v>18084570</v>
+        <v>13326219</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PELAYES</t>
+          <t>URRUTIA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>JOSE ALBERTO</t>
+          <t>MIGUEL ESTEBAN</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -7408,29 +7408,29 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1b</t>
+          <t>04. Caso CONFIRMADO de Infección por VHC</t>
         </is>
       </c>
       <c r="I75">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="J75">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>2020-22</t>
+          <t>2019-42</t>
         </is>
       </c>
       <c r="L75" s="2">
-        <v>44178</v>
+        <v>43754</v>
       </c>
       <c r="M75" s="3">
-        <v>43980</v>
+        <v>43753</v>
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>RIO GRANDE</t>
+          <t>USHUAIA</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -7455,42 +7455,42 @@
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="V75" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76">
-        <v>13326219</v>
+        <v>92825549</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>URRUTIA</t>
+          <t>NAIPIL BUSTOS</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>MIGUEL ESTEBAN</t>
+          <t>ALEJANDRO VLADIMIR</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7515,25 +7515,25 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>04. Caso CONFIRMADO de Infección por VHC</t>
+          <t>Virus Hepatitis C, genotipo 1a</t>
         </is>
       </c>
       <c r="I76">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J76">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>2019-42</t>
+          <t>2020-41</t>
         </is>
       </c>
       <c r="L76" s="2">
-        <v>43754</v>
+        <v>44178</v>
       </c>
       <c r="M76" s="3">
-        <v>43753</v>
+        <v>44109</v>
       </c>
       <c r="N76" t="inlineStr">
         <is>
@@ -7547,7 +7547,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>HIV</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -7588,16 +7588,16 @@
     </row>
     <row r="77">
       <c r="A77">
-        <v>92825549</v>
+        <v>17888898</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>NAIPIL BUSTOS</t>
+          <t>NIETO</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ALEJANDRO VLADIMIR</t>
+          <t>RAUL ENRIQUE</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7622,25 +7622,25 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1a</t>
+          <t>04. Caso CONFIRMADO de Infección por VHC</t>
         </is>
       </c>
       <c r="I77">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="J77">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>2020-41</t>
+          <t>2023-06</t>
         </is>
       </c>
       <c r="L77" s="2">
-        <v>44178</v>
+        <v>44972</v>
       </c>
       <c r="M77" s="3">
-        <v>44109</v>
+        <v>44963</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -7654,7 +7654,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>HIV</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -7695,16 +7695,16 @@
     </row>
     <row r="78">
       <c r="A78">
-        <v>17888898</v>
+        <v>14423827</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>NIETO</t>
+          <t>CANTERO</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>RAUL ENRIQUE</t>
+          <t>LUIS ALBERTO</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7729,29 +7729,29 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>04. Caso CONFIRMADO de Infección por VHC</t>
+          <t>Virus Hepatitis C, genotipo 1a</t>
         </is>
       </c>
       <c r="I78">
         <v>6</v>
       </c>
       <c r="J78">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>2023-06</t>
+          <t>2020-06</t>
         </is>
       </c>
       <c r="L78" s="2">
-        <v>44972</v>
+        <v>43865</v>
       </c>
       <c r="M78" s="3">
-        <v>44963</v>
+        <v>43865</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>USHUAIA</t>
+          <t>*SIN DATO* (*SIN DATO*)</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
@@ -7766,7 +7766,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7776,17 +7776,17 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="U78" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="V78" t="inlineStr">
@@ -7796,22 +7796,22 @@
       </c>
       <c r="W78" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79">
-        <v>14423827</v>
+        <v>14135708</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>CANTERO</t>
+          <t>PEREZ</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>LUIS ALBERTO</t>
+          <t>LAURA GLADYS</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7821,7 +7821,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -7836,29 +7836,29 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1a</t>
+          <t>Virus Hepatitis C, genotipo 1b</t>
         </is>
       </c>
       <c r="I79">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="J79">
         <v>2020</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>2020-06</t>
+          <t>2020-11</t>
         </is>
       </c>
       <c r="L79" s="2">
-        <v>43865</v>
+        <v>44178</v>
       </c>
       <c r="M79" s="3">
-        <v>43865</v>
+        <v>43902</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>*SIN DATO* (*SIN DATO*)</t>
+          <t>RIO GRANDE</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -7868,12 +7868,12 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>VHB</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7883,22 +7883,22 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="T79" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="U79" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="V79" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="W79" t="inlineStr">
@@ -7909,16 +7909,16 @@
     </row>
     <row r="80">
       <c r="A80">
-        <v>14135708</v>
+        <v>93633114</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PEREZ</t>
+          <t>PEREIRA PEREIRA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>LAURA GLADYS</t>
+          <t>JOSE ROBINSON</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7928,7 +7928,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -7943,25 +7943,25 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1b</t>
+          <t>03. Caso PROBABLE de Infección por VHC</t>
         </is>
       </c>
       <c r="I80">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="J80">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>2020-11</t>
+          <t>2023-05</t>
         </is>
       </c>
       <c r="L80" s="2">
-        <v>44178</v>
+        <v>45065</v>
       </c>
       <c r="M80" s="3">
-        <v>43902</v>
+        <v>44959</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
@@ -7970,62 +7970,27 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="P80" t="inlineStr">
-        <is>
-          <t>VHB</t>
-        </is>
-      </c>
-      <c r="Q80" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R80" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="S80" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="T80" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="U80" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="V80" t="inlineStr">
-        <is>
-          <t>SI</t>
+          <t>DESCARTADO</t>
         </is>
       </c>
       <c r="W80" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81">
-        <v>93633114</v>
+        <v>21816819</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PEREIRA PEREIRA</t>
+          <t>BARRIENTOS VIDAL</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>JOSE ROBINSON</t>
+          <t>LUIS GUILLERMO</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -8054,21 +8019,21 @@
         </is>
       </c>
       <c r="I81">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="J81">
         <v>2023</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>2023-05</t>
+          <t>2023-40</t>
         </is>
       </c>
       <c r="L81" s="2">
-        <v>45065</v>
+        <v>45247</v>
       </c>
       <c r="M81" s="3">
-        <v>44959</v>
+        <v>45204</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
@@ -8077,7 +8042,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>DESCARTADO</t>
+          <t>SIN DATOS</t>
         </is>
       </c>
       <c r="W81" t="inlineStr">
@@ -8088,26 +8053,26 @@
     </row>
     <row r="82">
       <c r="A82">
-        <v>21816819</v>
+        <v>27519553</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>BARRIENTOS VIDAL</t>
+          <t>VALDEZ</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO</t>
+          <t>PATRICIA MARGARITA</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>De 45 a 65 años</t>
+          <t>De 35 a 44 años</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -8126,21 +8091,21 @@
         </is>
       </c>
       <c r="I82">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="J82">
         <v>2023</v>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>2023-40</t>
+          <t>2023-11</t>
         </is>
       </c>
       <c r="L82" s="2">
-        <v>45247</v>
+        <v>45065</v>
       </c>
       <c r="M82" s="3">
-        <v>45204</v>
+        <v>45000</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
@@ -8160,21 +8125,21 @@
     </row>
     <row r="83">
       <c r="A83">
-        <v>27519553</v>
+        <v>25116055</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>VALDEZ</t>
+          <t>HOYOS</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>PATRICIA MARGARITA</t>
+          <t>FABIANA PATRICIA</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>De 35 a 44 años</t>
+          <t>De 45 a 65 años</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -8194,25 +8159,25 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>03. Caso PROBABLE de Infección por VHC</t>
+          <t>07. En estudio para Hepatitis C</t>
         </is>
       </c>
       <c r="I83">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="J83">
         <v>2023</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>2023-11</t>
+          <t>2023-44</t>
         </is>
       </c>
       <c r="L83" s="2">
-        <v>45065</v>
+        <v>45236</v>
       </c>
       <c r="M83" s="3">
-        <v>45000</v>
+        <v>45229</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
@@ -8232,26 +8197,26 @@
     </row>
     <row r="84">
       <c r="A84">
-        <v>25116055</v>
+        <v>34375222</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>HOYOS</t>
+          <t>MANCILLA MENDEZ</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>FABIANA PATRICIA</t>
+          <t>JORGE DAMIAN</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>De 45 a 65 años</t>
+          <t>De 35 a 44 años</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -8261,30 +8226,30 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Hepatitis virales</t>
+          <t>Banco de Sangre</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>07. En estudio para Hepatitis C</t>
+          <t>01. Caso probable en banco de sangre</t>
         </is>
       </c>
       <c r="I84">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="J84">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>2023-44</t>
+          <t>2025-49</t>
         </is>
       </c>
       <c r="L84" s="2">
-        <v>45236</v>
+        <v>46010</v>
       </c>
       <c r="M84" s="3">
-        <v>45229</v>
+        <v>45996</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
@@ -8304,21 +8269,21 @@
     </row>
     <row r="85">
       <c r="A85">
-        <v>34375222</v>
+        <v>22668469</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MANCILLA MENDEZ</t>
+          <t>RAMIREZ</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>JORGE DAMIAN</t>
+          <t>JULIO ARNALDO PABLO</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>De 35 a 44 años</t>
+          <t>De 45 a 65 años</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -8333,30 +8298,30 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Banco de Sangre</t>
+          <t>Hepatitis virales</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>01. Caso probable en banco de sangre</t>
+          <t>Virus Hepatitis C, genotipo 1a</t>
         </is>
       </c>
       <c r="I85">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="J85">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>2025-49</t>
+          <t>2023-44</t>
         </is>
       </c>
       <c r="L85" s="2">
-        <v>46010</v>
+        <v>45236</v>
       </c>
       <c r="M85" s="3">
-        <v>45996</v>
+        <v>45233</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -8365,27 +8330,62 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
           <t>SIN DATOS</t>
         </is>
       </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>SIN DATOS</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>SIN DATOS</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>SIN DATOS</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>SIN DATOS</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="W85" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86">
-        <v>22668469</v>
+        <v>17438241</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>RAMIREZ</t>
+          <t>SANTILLAN</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>JULIO ARNALDO PABLO</t>
+          <t>HECTOR EDUARDO</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -8410,25 +8410,25 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1a</t>
+          <t>Virus Hepatitis C, genotipo 1</t>
         </is>
       </c>
       <c r="I86">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="J86">
-        <v>2023</v>
+        <v>2019</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>2023-44</t>
+          <t>2019-31</t>
         </is>
       </c>
       <c r="L86" s="2">
-        <v>45236</v>
+        <v>43690</v>
       </c>
       <c r="M86" s="3">
-        <v>45233</v>
+        <v>43679</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -8447,52 +8447,52 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>SIN DATOS</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>SIN DATOS</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>SIN DATOS</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="T86" t="inlineStr">
         <is>
-          <t>SIN DATOS</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="U86" t="inlineStr">
         <is>
-          <t>SIN DATOS</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="V86" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="W86" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87">
-        <v>17438241</v>
+        <v>20066627</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SANTILLAN</t>
+          <t>MASI</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>HECTOR EDUARDO</t>
+          <t>CLAUDIA ESTER</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -8502,7 +8502,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -8517,25 +8517,25 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1</t>
+          <t>04. Caso CONFIRMADO de Infección por VHC</t>
         </is>
       </c>
       <c r="I87">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="J87">
         <v>2019</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>2019-31</t>
+          <t>2019-13</t>
         </is>
       </c>
       <c r="L87" s="2">
-        <v>43690</v>
+        <v>44923</v>
       </c>
       <c r="M87" s="3">
-        <v>43679</v>
+        <v>43550</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -8544,42 +8544,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="P87" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="Q87" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R87" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="S87" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="T87" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="U87" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="V87" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>DESCARTADO</t>
         </is>
       </c>
       <c r="W87" t="inlineStr">
@@ -8590,16 +8555,16 @@
     </row>
     <row r="88">
       <c r="A88">
-        <v>20066627</v>
+        <v>25006616</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MASI</t>
+          <t>PANIAGUA</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CLAUDIA ESTER</t>
+          <t>PAOLA</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -8624,25 +8589,25 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>04. Caso CONFIRMADO de Infección por VHC</t>
+          <t>Virus Hepatitis C, genotipo 1a</t>
         </is>
       </c>
       <c r="I88">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="J88">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>2019-13</t>
+          <t>2022-32</t>
         </is>
       </c>
       <c r="L88" s="2">
-        <v>44923</v>
+        <v>44932</v>
       </c>
       <c r="M88" s="3">
-        <v>43550</v>
+        <v>44781</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -8651,7 +8616,42 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>DESCARTADO</t>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="W88" t="inlineStr">
@@ -8662,16 +8662,16 @@
     </row>
     <row r="89">
       <c r="A89">
-        <v>25006616</v>
+        <v>13844552</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PANIAGUA</t>
+          <t>OVANDO</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>PAOLA</t>
+          <t>ROSA ESTHER</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -8696,7 +8696,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1a</t>
+          <t>Virus Hepatitis C, genotipo 1b</t>
         </is>
       </c>
       <c r="I89">
@@ -8711,14 +8711,14 @@
         </is>
       </c>
       <c r="L89" s="2">
-        <v>44932</v>
+        <v>44833</v>
       </c>
       <c r="M89" s="3">
-        <v>44781</v>
+        <v>44782</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>RIO GRANDE</t>
+          <t>USHUAIA</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -8753,7 +8753,7 @@
       </c>
       <c r="U89" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="V89" t="inlineStr">
@@ -8769,21 +8769,21 @@
     </row>
     <row r="90">
       <c r="A90">
-        <v>13844552</v>
+        <v>93744318</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>OVANDO</t>
+          <t>AGUILA AGUILA</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ROSA ESTHER</t>
+          <t>MIRNA ADELITA</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>De 45 a 65 años</t>
+          <t>Mayores de 65 años</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -8803,29 +8803,29 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1b</t>
+          <t>Virus Hepatitis C, genotipo 1a</t>
         </is>
       </c>
       <c r="I90">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="J90">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>2022-32</t>
+          <t>2025-50</t>
         </is>
       </c>
       <c r="L90" s="2">
-        <v>44833</v>
+        <v>46041</v>
       </c>
       <c r="M90" s="3">
-        <v>44782</v>
+        <v>46000</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>USHUAIA</t>
+          <t>RIO GRANDE</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
@@ -8840,7 +8840,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>Tto en curso</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8860,12 +8860,12 @@
       </c>
       <c r="U90" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>Tto en curso</t>
         </is>
       </c>
       <c r="V90" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="W90" t="inlineStr">
@@ -8876,21 +8876,21 @@
     </row>
     <row r="91">
       <c r="A91">
-        <v>93744318</v>
+        <v>94574916</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>AGUILA AGUILA</t>
+          <t>ROA RESQUIN</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>MIRNA ADELITA</t>
+          <t>NORMA ELIZABETH</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Mayores de 65 años</t>
+          <t>De 35 a 44 años</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -8910,25 +8910,25 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Virus Hepatitis C, genotipo 1a</t>
+          <t>05. Infección resuelta o falso anti VHC</t>
         </is>
       </c>
       <c r="I91">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="J91">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>2025-50</t>
+          <t>2024-32</t>
         </is>
       </c>
       <c r="L91" s="2">
-        <v>46041</v>
+        <v>45512</v>
       </c>
       <c r="M91" s="3">
-        <v>46000</v>
+        <v>45512</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
@@ -8937,42 +8937,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="P91" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="Q91" t="inlineStr">
-        <is>
-          <t>Tto en curso</t>
-        </is>
-      </c>
-      <c r="R91" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="S91" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="T91" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="U91" t="inlineStr">
-        <is>
-          <t>Tto en curso</t>
-        </is>
-      </c>
-      <c r="V91" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>DESCARTADO</t>
         </is>
       </c>
       <c r="W91" t="inlineStr">
@@ -8983,21 +8948,21 @@
     </row>
     <row r="92">
       <c r="A92">
-        <v>94574916</v>
+        <v>18265819</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ROA RESQUIN</t>
+          <t>VILLA</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>NORMA ELIZABETH</t>
+          <t>MARTA GLADYS</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>De 35 a 44 años</t>
+          <t>De 45 a 65 años</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -9017,25 +8982,25 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>05. Infección resuelta o falso anti VHC</t>
+          <t>04. Caso CONFIRMADO de Infección por VHC</t>
         </is>
       </c>
       <c r="I92">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="J92">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>2024-32</t>
+          <t>2025-14</t>
         </is>
       </c>
       <c r="L92" s="2">
-        <v>45512</v>
+        <v>45748</v>
       </c>
       <c r="M92" s="3">
-        <v>45512</v>
+        <v>45748</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
@@ -9044,7 +9009,42 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>DESCARTADO</t>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="W92" t="inlineStr">
@@ -9055,16 +9055,16 @@
     </row>
     <row r="93">
       <c r="A93">
-        <v>18265819</v>
+        <v>21970773</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VILLA</t>
+          <t>GARCIA</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>MARTA GLADYS</t>
+          <t>ROSA RAQUEL</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -9089,69 +9089,34 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>04. Caso CONFIRMADO de Infección por VHC</t>
+          <t>06. Caso DESCARTADO de Infección por VHC</t>
         </is>
       </c>
       <c r="I93">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="J93">
         <v>2025</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>2025-14</t>
+          <t>2025-35</t>
         </is>
       </c>
       <c r="L93" s="2">
-        <v>45748</v>
+        <v>45898</v>
       </c>
       <c r="M93" s="3">
-        <v>45748</v>
+        <v>45897</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>RIO GRANDE</t>
+          <t>USHUAIA</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="P93" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="Q93" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R93" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="S93" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="T93" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="U93" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="V93" t="inlineStr">
-        <is>
-          <t>NO</t>
+          <t>DESCARTADO</t>
         </is>
       </c>
       <c r="W93" t="inlineStr">
@@ -9162,16 +9127,16 @@
     </row>
     <row r="94">
       <c r="A94">
-        <v>21970773</v>
+        <v>20853965</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>GARCIA</t>
+          <t>BRUNO</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ROSA RAQUEL</t>
+          <t>MARCELO FABIAN</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -9181,7 +9146,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -9196,25 +9161,25 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>06. Caso DESCARTADO de Infección por VHC</t>
+          <t>04. Caso CONFIRMADO de Infección por VHC</t>
         </is>
       </c>
       <c r="I94">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="J94">
-        <v>2025</v>
+        <v>2019</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>2025-35</t>
+          <t>2019-38</t>
         </is>
       </c>
       <c r="L94" s="2">
-        <v>45898</v>
+        <v>43754</v>
       </c>
       <c r="M94" s="3">
-        <v>45897</v>
+        <v>43724</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
@@ -9223,7 +9188,42 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>DESCARTADO</t>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="W94" t="inlineStr">
@@ -9234,16 +9234,16 @@
     </row>
     <row r="95">
       <c r="A95">
-        <v>20853965</v>
+        <v>12693857</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>BRUNO</t>
+          <t>ORTIZ</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>MARCELO FABIAN</t>
+          <t>OLGA BEATRIZ</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -9253,7 +9253,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -9268,69 +9268,34 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>04. Caso CONFIRMADO de Infección por VHC</t>
+          <t>03. Caso PROBABLE de Infección por VHC</t>
         </is>
       </c>
       <c r="I95">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="J95">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>2019-38</t>
+          <t>2018-52</t>
         </is>
       </c>
       <c r="L95" s="2">
-        <v>43754</v>
+        <v>43503</v>
       </c>
       <c r="M95" s="3">
-        <v>43724</v>
+        <v>43461</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>USHUAIA</t>
+          <t>RIO GRANDE</t>
         </is>
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="P95" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="Q95" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R95" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="S95" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="T95" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="U95" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="V95" t="inlineStr">
-        <is>
-          <t>SI</t>
+          <t>DESCARTADO</t>
         </is>
       </c>
       <c r="W95" t="inlineStr">
@@ -9341,26 +9306,26 @@
     </row>
     <row r="96">
       <c r="A96">
-        <v>12693857</v>
+        <v>34423562</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ORTIZ</t>
+          <t>GASC</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>OLGA BEATRIZ</t>
+          <t>MARIO LEONARDO</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>De 45 a 65 años</t>
+          <t>De 25 a 34 años</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -9379,30 +9344,30 @@
         </is>
       </c>
       <c r="I96">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="J96">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>2018-52</t>
+          <t>2020-29</t>
         </is>
       </c>
       <c r="L96" s="2">
-        <v>43503</v>
+        <v>44176</v>
       </c>
       <c r="M96" s="3">
-        <v>43461</v>
+        <v>44027</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>RIO GRANDE</t>
+          <t>TOLHUIN</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>DESCARTADO</t>
+          <t>SIN DATOS</t>
         </is>
       </c>
       <c r="W96" t="inlineStr">
@@ -9413,21 +9378,21 @@
     </row>
     <row r="97">
       <c r="A97">
-        <v>34423562</v>
+        <v>8599406</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>GASC</t>
+          <t>ARSELLI</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>MARIO LEONARDO</t>
+          <t>ARMANDO RICARDO</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>De 25 a 34 años</t>
+          <t>Mayores de 65 años</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -9447,25 +9412,25 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>03. Caso PROBABLE de Infección por VHC</t>
+          <t>04. Caso CONFIRMADO de Infección por VHC</t>
         </is>
       </c>
       <c r="I97">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J97">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>2020-29</t>
+          <t>2024-27</t>
         </is>
       </c>
       <c r="L97" s="2">
-        <v>44176</v>
+        <v>45478</v>
       </c>
       <c r="M97" s="3">
-        <v>44027</v>
+        <v>45476</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
@@ -9474,7 +9439,42 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
           <t>SIN DATOS</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>SIN DATOS</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="W97" t="inlineStr">
@@ -9485,21 +9485,21 @@
     </row>
     <row r="98">
       <c r="A98">
-        <v>8599406</v>
+        <v>33099926</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ARSELLI</t>
+          <t>VILCA</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ARMANDO RICARDO</t>
+          <t>DENIS LEONEL</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Mayores de 65 años</t>
+          <t>De 35 a 44 años</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -9523,65 +9523,30 @@
         </is>
       </c>
       <c r="I98">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="J98">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>2024-27</t>
+          <t>2022-02</t>
         </is>
       </c>
       <c r="L98" s="2">
-        <v>45478</v>
+        <v>44932</v>
       </c>
       <c r="M98" s="3">
-        <v>45476</v>
+        <v>44573</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>TOLHUIN</t>
+          <t>USHUAIA</t>
         </is>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="P98" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="Q98" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R98" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="S98" t="inlineStr">
-        <is>
           <t>SIN DATOS</t>
-        </is>
-      </c>
-      <c r="T98" t="inlineStr">
-        <is>
-          <t>SIN DATOS</t>
-        </is>
-      </c>
-      <c r="U98" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="V98" t="inlineStr">
-        <is>
-          <t>SI</t>
         </is>
       </c>
       <c r="W98" t="inlineStr">
@@ -9592,21 +9557,21 @@
     </row>
     <row r="99">
       <c r="A99">
-        <v>33099926</v>
+        <v>33845183</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>VILCA</t>
+          <t>MORA</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>DENIS LEONEL</t>
+          <t>SERGIO ORLANDO</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>De 35 a 44 años</t>
+          <t>De 25 a 34 años</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -9630,21 +9595,21 @@
         </is>
       </c>
       <c r="I99">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="J99">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>2022-02</t>
+          <t>2023-16</t>
         </is>
       </c>
       <c r="L99" s="2">
-        <v>44932</v>
+        <v>45240</v>
       </c>
       <c r="M99" s="3">
-        <v>44573</v>
+        <v>45033</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -9653,117 +9618,45 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>SIN DATOS</t>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>HIV</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="W99" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100">
-        <v>33845183</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>MORA</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>SERGIO ORLANDO</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>De 25 a 34 años</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>Hepatitis C</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>Hepatitis virales</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>04. Caso CONFIRMADO de Infección por VHC</t>
-        </is>
-      </c>
-      <c r="I100">
-        <v>16</v>
-      </c>
-      <c r="J100">
-        <v>2023</v>
-      </c>
-      <c r="K100" t="inlineStr">
-        <is>
-          <t>2023-16</t>
-        </is>
-      </c>
-      <c r="L100" s="2">
-        <v>45240</v>
-      </c>
-      <c r="M100" s="3">
-        <v>45033</v>
-      </c>
-      <c r="N100" t="inlineStr">
-        <is>
-          <t>USHUAIA</t>
-        </is>
-      </c>
-      <c r="O100" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="P100" t="inlineStr">
-        <is>
-          <t>HIV</t>
-        </is>
-      </c>
-      <c r="Q100" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R100" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="S100" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="T100" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="U100" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="V100" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="W100" t="inlineStr">
         <is>
           <t>NO</t>
         </is>

</xml_diff>